<commit_message>
docs: update hardware inventory with 2026 survey findings. Work in progress (extends Gael's 2025 work)
</commit_message>
<xml_diff>
--- a/Docs/IDMIL_T-Sticks.xlsx
+++ b/Docs/IDMIL_T-Sticks.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gaelm\Documents\Projets\T-Stick\IDMIL\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alexnieva\projects\tstick-dev\firmware\T-Stick\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2952928A-5097-4ADA-853A-ECDC1B404159}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0267EC2A-1F35-4B1F-9EC9-04C7B8E45A7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata">
   <metadataTypes count="1">
     <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
   </metadataTypes>
@@ -188,7 +188,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="36">
   <si>
     <t>Update:</t>
   </si>
@@ -234,12 +234,6 @@
     <t>Last Review</t>
   </si>
   <si>
-    <t>turns on as 001
-flow of OSC messages very slow ~1/s
-button and switch don't seem to do anything
-works only when plugged</t>
-  </si>
-  <si>
     <t>Soprano</t>
   </si>
   <si>
@@ -285,6 +279,34 @@
     <t>USB connection is loose
 need reflash?
 Needs to be plugged to work</t>
+  </si>
+  <si>
+    <t>2G</t>
+  </si>
+  <si>
+    <t>with Alex Nieva</t>
+  </si>
+  <si>
+    <t>31-07-2026</t>
+  </si>
+  <si>
+    <t>Seems to have a TinyPico USB-C from Adafruit. TBC. Not tested</t>
+  </si>
+  <si>
+    <t>turns on as 001. Stopped working. Alex opened.
+Hacked for haptics tests. Has two DRV2605L boards for voice coils. Lolin D32+capsense+LSM9DS1 Sparkfun</t>
+  </si>
+  <si>
+    <t>19X</t>
+  </si>
+  <si>
+    <t>Lolin D32+capsense LSM9DS1 from Adafruit+ Piezo+3.7 flat battery. Not working</t>
+  </si>
+  <si>
+    <t>First Sopranino Wired from 2017. https://github.com/alexnieva/T-Stick/tree/master/Sopranino/2G/172</t>
+  </si>
+  <si>
+    <t>Enchanti+trill. Works</t>
   </si>
 </sst>
 </file>
@@ -338,7 +360,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
@@ -364,11 +386,20 @@
     <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -779,30 +810,30 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J20"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:J23"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.5546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.88671875" style="1"/>
-    <col min="5" max="5" width="10.77734375" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="50.77734375" style="2" customWidth="1"/>
-    <col min="7" max="8" width="16.77734375" style="2" customWidth="1"/>
-    <col min="9" max="9" width="48.77734375" style="1" customWidth="1"/>
-    <col min="10" max="10" width="16.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.5703125" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.85546875" style="1"/>
+    <col min="5" max="5" width="10.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="50.7109375" style="2" customWidth="1"/>
+    <col min="7" max="8" width="16.7109375" style="2" customWidth="1"/>
+    <col min="9" max="9" width="48.7109375" style="1" customWidth="1"/>
+    <col min="10" max="10" width="16.140625" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="10">
+      <c r="B1" s="9">
         <f ca="1">TODAY()</f>
-        <v>45727</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>46234</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
         <v>1</v>
       </c>
@@ -818,61 +849,73 @@
       <c r="E4" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="F4" s="9" t="s">
+      <c r="F4" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="G4" s="9"/>
-      <c r="H4" s="9"/>
+      <c r="G4" s="10"/>
+      <c r="H4" s="10"/>
       <c r="I4" s="5" t="s">
         <v>5</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" ht="64.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="3">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" s="12" customFormat="1" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="11">
+        <v>172</v>
+      </c>
+      <c r="B5" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D5" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="F5" s="11"/>
+      <c r="G5" s="11"/>
+      <c r="H5" s="11"/>
+      <c r="I5" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="J5" s="11" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" s="12" customFormat="1" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="B6" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6" s="11">
+        <v>4</v>
+      </c>
+      <c r="D6" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="F6" s="11"/>
+      <c r="G6" s="11"/>
+      <c r="H6" s="11"/>
+      <c r="I6" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="J6" s="11" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="64.150000000000006" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="3">
         <v>191</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="J5" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" ht="64.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="3">
-        <v>193</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C6" s="3">
-        <v>4</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="F6" s="6" t="e" vm="1">
-        <v>#VALUE!</v>
-      </c>
-      <c r="G6" s="2" t="e" vm="2">
-        <v>#VALUE!</v>
-      </c>
-      <c r="H6" s="2" t="e" vm="3">
-        <v>#VALUE!</v>
-      </c>
-      <c r="I6" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="J6" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" ht="64.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="3">
-        <v>194</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>6</v>
@@ -883,28 +926,19 @@
       <c r="D7" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="E7" s="8">
-        <v>45535</v>
-      </c>
-      <c r="F7" s="2" t="e" vm="4">
-        <v>#VALUE!</v>
-      </c>
-      <c r="G7" s="2" t="e" vm="5">
-        <v>#VALUE!</v>
-      </c>
-      <c r="H7" s="2" t="e" vm="6">
-        <v>#VALUE!</v>
+      <c r="E7" s="1" t="s">
+        <v>29</v>
       </c>
       <c r="I7" s="7" t="s">
-        <v>9</v>
+        <v>30</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" ht="64.05" customHeight="1" x14ac:dyDescent="0.3">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="64.150000000000006" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3">
-        <v>308</v>
+        <v>193</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>6</v>
@@ -915,28 +949,28 @@
       <c r="D8" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="E8" s="8">
-        <v>45535</v>
-      </c>
-      <c r="F8" s="2" t="e" vm="7">
-        <v>#VALUE!</v>
-      </c>
-      <c r="G8" s="2" t="e" vm="8">
-        <v>#VALUE!</v>
-      </c>
-      <c r="H8" s="2" t="e" vm="9">
+      <c r="E8" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="F8" s="6" t="e" vm="1">
+        <v>#VALUE!</v>
+      </c>
+      <c r="G8" s="2" t="e" vm="2">
+        <v>#VALUE!</v>
+      </c>
+      <c r="H8" s="2" t="e" vm="3">
         <v>#VALUE!</v>
       </c>
       <c r="I8" s="7" t="s">
-        <v>10</v>
+        <v>31</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" ht="64.05" customHeight="1" x14ac:dyDescent="0.3">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="64.150000000000006" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3">
-        <v>311</v>
+        <v>194</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>6</v>
@@ -947,90 +981,120 @@
       <c r="D9" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="F9" s="2" t="e" vm="10">
-        <v>#VALUE!</v>
-      </c>
-      <c r="G9" s="2" t="e" vm="11">
-        <v>#VALUE!</v>
-      </c>
-      <c r="H9" s="2" t="e" vm="12">
-        <v>#VALUE!</v>
+      <c r="E9" s="8">
+        <v>45535</v>
+      </c>
+      <c r="F9" s="2" t="e" vm="4">
+        <v>#VALUE!</v>
+      </c>
+      <c r="G9" s="2" t="e" vm="5">
+        <v>#VALUE!</v>
+      </c>
+      <c r="H9" s="2" t="e" vm="6">
+        <v>#VALUE!</v>
+      </c>
+      <c r="I9" s="7" t="s">
+        <v>9</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" ht="64.05" customHeight="1" x14ac:dyDescent="0.3">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="64.150000000000006" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3">
+        <v>308</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C10" s="3">
+        <v>4</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E10" s="8">
+        <v>45535</v>
+      </c>
+      <c r="F10" s="2" t="e" vm="7">
+        <v>#VALUE!</v>
+      </c>
+      <c r="G10" s="2" t="e" vm="8">
+        <v>#VALUE!</v>
+      </c>
+      <c r="H10" s="2" t="e" vm="9">
+        <v>#VALUE!</v>
+      </c>
+      <c r="I10" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="J10" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="64.150000000000006" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="3">
+        <v>311</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C11" s="3">
+        <v>4</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F11" s="2" t="e" vm="10">
+        <v>#VALUE!</v>
+      </c>
+      <c r="G11" s="2" t="e" vm="11">
+        <v>#VALUE!</v>
+      </c>
+      <c r="H11" s="2" t="e" vm="12">
+        <v>#VALUE!</v>
+      </c>
+      <c r="J11" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="64.150000000000006" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="3">
         <v>315</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B12" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C12" s="3" t="s">
         <v>14</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="I10" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="J10" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" ht="64.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="3">
-        <v>500</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C11" s="3">
-        <v>5</v>
-      </c>
-      <c r="I11" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="J11" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" ht="64.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="3">
-        <v>514</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C12" s="3">
-        <v>5</v>
-      </c>
-      <c r="F12" s="2" t="e" vm="13">
-        <v>#VALUE!</v>
-      </c>
-      <c r="G12" s="2" t="e" vm="14">
-        <v>#VALUE!</v>
       </c>
       <c r="I12" s="7" t="s">
         <v>26</v>
       </c>
       <c r="J12" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="64.150000000000006" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="3">
+        <v>500</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C13" s="3">
+        <v>5</v>
+      </c>
+      <c r="I13" s="7" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="13" spans="1:10" ht="64.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="3">
-        <v>516</v>
-      </c>
-      <c r="I13" s="7" t="s">
-        <v>20</v>
-      </c>
       <c r="J13" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" ht="64.05" customHeight="1" x14ac:dyDescent="0.3">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="64.150000000000006" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3">
-        <v>517</v>
+        <v>514</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>6</v>
@@ -1038,33 +1102,33 @@
       <c r="C14" s="3">
         <v>5</v>
       </c>
-      <c r="I14" s="1" t="s">
-        <v>16</v>
+      <c r="F14" s="2" t="e" vm="13">
+        <v>#VALUE!</v>
+      </c>
+      <c r="G14" s="2" t="e" vm="14">
+        <v>#VALUE!</v>
+      </c>
+      <c r="I14" s="7" t="s">
+        <v>25</v>
       </c>
       <c r="J14" s="1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" ht="64.05" customHeight="1" x14ac:dyDescent="0.3">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="64.150000000000006" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3">
-        <v>555</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C15" s="3">
-        <v>5</v>
-      </c>
-      <c r="I15" s="1" t="s">
+        <v>516</v>
+      </c>
+      <c r="I15" s="7" t="s">
         <v>19</v>
       </c>
       <c r="J15" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" ht="64.05" customHeight="1" x14ac:dyDescent="0.3">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" ht="64.150000000000006" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3">
-        <v>566</v>
+        <v>517</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>6</v>
@@ -1073,15 +1137,15 @@
         <v>5</v>
       </c>
       <c r="I16" s="1" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="J16" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" ht="64.05" customHeight="1" x14ac:dyDescent="0.3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" ht="64.150000000000006" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3">
-        <v>569</v>
+        <v>555</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>6</v>
@@ -1093,22 +1157,76 @@
         <v>18</v>
       </c>
       <c r="J17" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" ht="64.05" customHeight="1" x14ac:dyDescent="0.3">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" ht="64.150000000000006" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="3">
+        <v>566</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C18" s="3">
+        <v>5</v>
+      </c>
+      <c r="I18" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="J18" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" ht="64.150000000000006" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="3">
+        <v>569</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C19" s="3">
+        <v>5</v>
+      </c>
+      <c r="I19" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="J19" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" ht="64.150000000000006" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="3">
+        <v>571</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C20" s="3">
+        <v>5</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="I20" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="J20" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" ht="64.150000000000006" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="3">
         <v>588</v>
       </c>
-      <c r="I18" s="1" t="s">
+      <c r="I21" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="J18" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" ht="64.05" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="20" spans="1:10" ht="64.05" customHeight="1" x14ac:dyDescent="0.3"/>
+      <c r="J21" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" ht="64.150000000000006" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="23" spans="1:10" ht="64.150000000000006" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="F4:H4"/>

</xml_diff>